<commit_message>
correção busca de pedidos
</commit_message>
<xml_diff>
--- a/utils/Modelos Importação/preenchido/Programação - Pedido - Item - MJPD0401.xlsx
+++ b/utils/Modelos Importação/preenchido/Programação - Pedido - Item - MJPD0401.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Odeclei\Projeto James\01 - Teste Apontamento Produção\Apontamento Produção 4.0\utils\Modelos Importação\preenchido\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{607E08DB-C8BD-4DBF-BC31-784BBE9AF94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A40A363F-FEE3-47DA-8132-63D1DC06037D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="27510" windowHeight="16440" xr2:uid="{95162B4D-7AD8-4BD1-AC78-F7AF31A241AA}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="403">
   <si>
     <t>PROGRAMAÇÃO</t>
   </si>
@@ -1199,6 +1199,36 @@
   </si>
   <si>
     <t>OBS_PEDIDO</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>189871</t>
+  </si>
+  <si>
+    <t>189895</t>
+  </si>
+  <si>
+    <t>189907</t>
+  </si>
+  <si>
+    <t>3650</t>
+  </si>
+  <si>
+    <t>3655</t>
+  </si>
+  <si>
+    <t>3661</t>
+  </si>
+  <si>
+    <t>19728</t>
+  </si>
+  <si>
+    <t>19726</t>
   </si>
 </sst>
 </file>
@@ -5086,8 +5116,8 @@
       <c r="C130" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="D130" s="1">
-        <v>189979</v>
+      <c r="D130" s="1" t="s">
+        <v>390</v>
       </c>
       <c r="E130" s="4" t="s">
         <v>210</v>
@@ -5109,8 +5139,8 @@
       <c r="C131" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="D131" s="1">
-        <v>189979</v>
+      <c r="D131" s="1" t="s">
+        <v>390</v>
       </c>
       <c r="E131" s="4" t="s">
         <v>212</v>
@@ -5132,8 +5162,8 @@
       <c r="C132" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="D132" s="1">
-        <v>123</v>
+      <c r="D132" s="1" t="s">
+        <v>393</v>
       </c>
       <c r="E132" s="4" t="s">
         <v>215</v>
@@ -5155,8 +5185,8 @@
       <c r="C133" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="D133" s="1">
-        <v>123</v>
+      <c r="D133" s="1" t="s">
+        <v>393</v>
       </c>
       <c r="E133" s="4" t="s">
         <v>217</v>
@@ -5178,8 +5208,8 @@
       <c r="C134" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="D134" s="1">
-        <v>123</v>
+      <c r="D134" s="1" t="s">
+        <v>393</v>
       </c>
       <c r="E134" s="4" t="s">
         <v>219</v>
@@ -5224,8 +5254,8 @@
       <c r="C136" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="D136" s="1">
-        <v>45</v>
+      <c r="D136" s="1" t="s">
+        <v>394</v>
       </c>
       <c r="E136" s="4" t="s">
         <v>225</v>
@@ -5316,8 +5346,8 @@
       <c r="C140" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="D140" s="1">
-        <v>189871</v>
+      <c r="D140" s="1" t="s">
+        <v>395</v>
       </c>
       <c r="E140" s="4" t="s">
         <v>232</v>
@@ -5339,8 +5369,8 @@
       <c r="C141" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="D141" s="1">
-        <v>189871</v>
+      <c r="D141" s="1" t="s">
+        <v>395</v>
       </c>
       <c r="E141" s="4" t="s">
         <v>234</v>
@@ -5362,8 +5392,8 @@
       <c r="C142" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D142" s="1">
-        <v>189895</v>
+      <c r="D142" s="1" t="s">
+        <v>396</v>
       </c>
       <c r="E142" s="4" t="s">
         <v>217</v>
@@ -5385,8 +5415,8 @@
       <c r="C143" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D143" s="1">
-        <v>189895</v>
+      <c r="D143" s="1" t="s">
+        <v>396</v>
       </c>
       <c r="E143" s="4" t="s">
         <v>215</v>
@@ -5408,8 +5438,8 @@
       <c r="C144" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D144" s="1">
-        <v>189907</v>
+      <c r="D144" s="1" t="s">
+        <v>397</v>
       </c>
       <c r="E144" s="4" t="s">
         <v>223</v>
@@ -5431,8 +5461,8 @@
       <c r="C145" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="D145" s="1">
-        <v>3650</v>
+      <c r="D145" s="1" t="s">
+        <v>398</v>
       </c>
       <c r="E145" s="4" t="s">
         <v>223</v>
@@ -5454,8 +5484,8 @@
       <c r="C146" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="D146" s="1">
-        <v>3655</v>
+      <c r="D146" s="1" t="s">
+        <v>399</v>
       </c>
       <c r="E146" s="4" t="s">
         <v>223</v>
@@ -5477,8 +5507,8 @@
       <c r="C147" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D147" s="1">
-        <v>3661</v>
+      <c r="D147" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="E147" s="4" t="s">
         <v>232</v>
@@ -5500,8 +5530,8 @@
       <c r="C148" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D148" s="1">
-        <v>3661</v>
+      <c r="D148" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="E148" s="4" t="s">
         <v>219</v>
@@ -5523,8 +5553,8 @@
       <c r="C149" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D149" s="1">
-        <v>3661</v>
+      <c r="D149" s="1" t="s">
+        <v>400</v>
       </c>
       <c r="E149" s="4" t="s">
         <v>223</v>
@@ -5546,8 +5576,8 @@
       <c r="C150" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="D150" s="1">
-        <v>19728</v>
+      <c r="D150" s="1" t="s">
+        <v>401</v>
       </c>
       <c r="E150" s="4" t="s">
         <v>234</v>
@@ -5638,8 +5668,8 @@
       <c r="C154" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="D154" s="1">
-        <v>19726</v>
+      <c r="D154" s="1" t="s">
+        <v>402</v>
       </c>
       <c r="E154" s="4" t="s">
         <v>234</v>

</xml_diff>